<commit_message>
Update Excel sample file
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exel/Mẫu xuống xe.xlsx
+++ b/exel/Mẫu xuống xe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\NLChanhthu-main\exel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B3267C-C768-4CE6-A1E5-51C21C28E2A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2A490AC-6ACA-4BA5-9798-690BA07BC84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -702,7 +702,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -742,34 +742,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -845,12 +819,23 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
         <color rgb="FF000000"/>
-      </right>
-      <top/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -875,14 +860,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -918,10 +895,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -959,38 +932,38 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="4" fillId="5" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1012,11 +985,11 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1028,32 +1001,17 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="11" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="22" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1068,7 +1026,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1078,35 +1036,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1117,6 +1072,31 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1556,8 +1536,8 @@
   <dimension ref="A1:P31"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="20" customWidth="1"/>
-    <col min="2" max="2" width="21.109375" style="20" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="18" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" style="18" customWidth="1"/>
     <col min="3" max="3" width="39.109375" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="19.88671875" customWidth="1"/>
@@ -1570,37 +1550,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="70.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="19"/>
-      <c r="B1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-    </row>
-    <row r="2" spans="1:16" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="91" t="s">
+      <c r="A1" s="17"/>
+      <c r="B1" s="82" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+    </row>
+    <row r="2" spans="1:16" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
       <c r="J2"/>
       <c r="K2"/>
       <c r="L2"/>
@@ -1609,482 +1589,482 @@
       <c r="O2"/>
     </row>
     <row r="3" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72">
+      <c r="B3" s="65">
         <f ca="1">'CHI TIET'!M4</f>
-        <v>46287.616093055556</v>
+        <v>46297.399875578703</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="12">
         <f>'CHI TIET'!M5</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="63" t="str">
+      <c r="B4" s="60" t="str">
         <f>'CHI TIET'!C5</f>
         <v>66A-481.96</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="50">
+      <c r="F4" s="47">
         <f>E25</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="37"/>
-      <c r="B5" s="37"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
       <c r="E5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="48" t="e">
+      <c r="F5" s="45" t="e">
         <f>1-(F3/F4)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H5" s="47"/>
-    </row>
-    <row r="6" spans="1:16" s="32" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
+      <c r="H5" s="44"/>
+    </row>
+    <row r="6" spans="1:16" s="29" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="46" t="s">
+      <c r="E6" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="46" t="s">
+      <c r="F6" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="39">
+      <c r="A7" s="36">
         <v>1</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="51">
+      <c r="E7" s="48">
         <f>'CHI TIET'!C83</f>
         <v>0</v>
       </c>
-      <c r="F7" s="39"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="39">
+      <c r="A8" s="36">
         <v>2</v>
       </c>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="48">
         <f>'CHI TIET'!F82</f>
         <v>0</v>
       </c>
-      <c r="F8" s="39"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="39">
+      <c r="A9" s="36">
         <v>3</v>
       </c>
-      <c r="B9" s="40" t="s">
+      <c r="B9" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="48">
         <f>'CHI TIET'!C84</f>
         <v>0</v>
       </c>
-      <c r="F9" s="39"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
     </row>
     <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="39">
+      <c r="A10" s="36">
         <v>4</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="51">
+      <c r="E10" s="48">
         <f>'CHI TIET'!F83</f>
         <v>0</v>
       </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
     </row>
     <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="39">
+      <c r="A11" s="36">
         <v>5</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="41" t="s">
+      <c r="C11" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="51">
+      <c r="E11" s="48">
         <f>'CHI TIET'!F84</f>
         <v>0</v>
       </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
     </row>
     <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="39">
+      <c r="A12" s="36">
         <v>6</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="41" t="s">
+      <c r="B12" s="36"/>
+      <c r="C12" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="39" t="s">
+      <c r="D12" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="51">
+      <c r="E12" s="48">
         <f>'CHI TIET'!C82</f>
         <v>0</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
     </row>
     <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="39">
+      <c r="A13" s="36">
         <v>7</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="51">
+      <c r="E13" s="48">
         <f>'CHI TIET'!I78</f>
         <v>0</v>
       </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
     </row>
     <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="39">
+      <c r="A14" s="36">
         <v>8</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="51">
+      <c r="E14" s="48">
         <f>'CHI TIET'!I79</f>
         <v>0</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
     </row>
     <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="39">
+      <c r="A15" s="36">
         <v>9</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="41" t="s">
+      <c r="C15" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="51">
+      <c r="E15" s="48">
         <f>'CHI TIET'!C79</f>
         <v>0</v>
       </c>
-      <c r="F15" s="39"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
     </row>
     <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="39">
+      <c r="A16" s="36">
         <v>10</v>
       </c>
-      <c r="B16" s="40" t="s">
+      <c r="B16" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="41" t="s">
+      <c r="C16" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="51">
+      <c r="E16" s="48">
         <f>'CHI TIET'!F78</f>
         <v>0</v>
       </c>
-      <c r="F16" s="39"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
     </row>
     <row r="17" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="39">
+      <c r="A17" s="36">
         <v>11</v>
       </c>
-      <c r="B17" s="40" t="s">
+      <c r="B17" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="C17" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="51">
+      <c r="E17" s="48">
         <f>'CHI TIET'!C80</f>
         <v>0</v>
       </c>
-      <c r="F17" s="39"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
     </row>
     <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="39">
+      <c r="A18" s="36">
         <v>12</v>
       </c>
-      <c r="B18" s="40" t="s">
+      <c r="B18" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="41" t="s">
+      <c r="C18" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="51">
+      <c r="E18" s="48">
         <f>'CHI TIET'!F79</f>
         <v>0</v>
       </c>
-      <c r="F18" s="39"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
     </row>
     <row r="19" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="39">
+      <c r="A19" s="36">
         <v>13</v>
       </c>
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="41" t="s">
+      <c r="C19" s="38" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="39" t="s">
+      <c r="D19" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="51">
+      <c r="E19" s="48">
         <f>'CHI TIET'!F80</f>
         <v>0</v>
       </c>
-      <c r="F19" s="39"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
     </row>
     <row r="20" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="39">
+      <c r="A20" s="36">
         <v>14</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="41" t="s">
+      <c r="B20" s="36"/>
+      <c r="C20" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="51">
+      <c r="E20" s="48">
         <f>'CHI TIET'!C78</f>
         <v>0</v>
       </c>
-      <c r="F20" s="39" t="s">
+      <c r="F20" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
     </row>
     <row r="21" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="39">
+      <c r="A21" s="36">
         <v>15</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="52">
+      <c r="E21" s="49">
         <f>'CHI TIET'!C87</f>
         <v>0</v>
       </c>
-      <c r="F21" s="42"/>
+      <c r="F21" s="39"/>
     </row>
     <row r="22" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="39">
+      <c r="A22" s="36">
         <v>16</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="51">
+      <c r="E22" s="48">
         <f>'CHI TIET'!C88</f>
         <v>0</v>
       </c>
-      <c r="F22" s="42"/>
+      <c r="F22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="39">
+      <c r="A23" s="36">
         <v>17</v>
       </c>
-      <c r="B23" s="41" t="s">
+      <c r="B23" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="51">
+      <c r="E23" s="48">
         <f>'CHI TIET'!C85</f>
         <v>0</v>
       </c>
-      <c r="F23" s="42"/>
+      <c r="F23" s="39"/>
     </row>
     <row r="24" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="39">
+      <c r="A24" s="36">
         <v>18</v>
       </c>
-      <c r="B24" s="41" t="s">
+      <c r="B24" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="51">
+      <c r="E24" s="48">
         <f>'CHI TIET'!F85</f>
         <v>0</v>
       </c>
-      <c r="F24" s="42"/>
+      <c r="F24" s="39"/>
     </row>
     <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="43"/>
-      <c r="B25" s="87" t="s">
+      <c r="A25" s="40"/>
+      <c r="B25" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="88"/>
-      <c r="D25" s="89"/>
-      <c r="E25" s="44">
+      <c r="C25" s="80"/>
+      <c r="D25" s="81"/>
+      <c r="E25" s="41">
         <f>SUM(E7:E22)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="45"/>
+      <c r="F25" s="42"/>
     </row>
     <row r="31" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="33" t="s">
+      <c r="C31" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="F31" s="33" t="s">
+      <c r="F31" s="30" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2112,8 +2092,8 @@
   <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" style="20" customWidth="1"/>
-    <col min="2" max="2" width="21.109375" style="20" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" style="18" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" style="18" customWidth="1"/>
     <col min="3" max="3" width="39.109375" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="19.88671875" customWidth="1"/>
@@ -2131,37 +2111,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="70.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="19"/>
-      <c r="B1" s="90" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-    </row>
-    <row r="2" spans="1:16" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
+      <c r="A1" s="17"/>
+      <c r="B1" s="82" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="15"/>
+    </row>
+    <row r="2" spans="1:16" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
       <c r="J2"/>
       <c r="K2"/>
       <c r="L2"/>
@@ -2170,320 +2150,320 @@
       <c r="O2"/>
     </row>
     <row r="3" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72">
+      <c r="B3" s="65">
         <f ca="1">'CHI TIET'!M4</f>
-        <v>46287.616093055556</v>
-      </c>
-      <c r="E3" s="73" t="s">
+        <v>46297.399875578703</v>
+      </c>
+      <c r="E3" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="12">
         <f>'CHI TIET'!M5</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="66" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="74" t="str">
+      <c r="B4" s="67" t="str">
         <f>'CHI TIET'!C5</f>
         <v>66A-481.96</v>
       </c>
-      <c r="E4" s="73" t="s">
+      <c r="E4" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="50" t="e" vm="1">
+      <c r="F4" s="47" t="e" vm="1">
         <f>E23</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="66" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="75" t="str">
+      <c r="B5" s="68" t="str">
         <f>MID('CHI TIET'!D6,7,8)</f>
         <v/>
       </c>
-      <c r="E5" s="73" t="s">
+      <c r="E5" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="48" t="e" vm="1">
+      <c r="F5" s="45" t="e" vm="1">
         <f>1-(F3/F4)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H5" s="47"/>
-    </row>
-    <row r="6" spans="1:16" s="32" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
+      <c r="H5" s="44"/>
+    </row>
+    <row r="6" spans="1:16" s="29" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="46" t="s">
+      <c r="E6" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="46" t="s">
+      <c r="F6" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
     </row>
     <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="39">
+      <c r="A7" s="36">
         <v>1</v>
       </c>
-      <c r="B7" s="40" t="e" cm="1" vm="2">
+      <c r="B7" s="37" t="e" cm="1" vm="2">
         <f t="array" ref="B7">_xlfn._xlws.FILTER('TẤT CẢ'!B7:B24, ('TẤT CẢ'!E7:E24&lt;&gt;0) * ('TẤT CẢ'!E7:E24&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="C7" s="40" t="e" cm="1" vm="2">
+      <c r="C7" s="37" t="e" cm="1" vm="2">
         <f t="array" ref="C7">_xlfn._xlws.FILTER('TẤT CẢ'!C7:C24, ('TẤT CẢ'!E7:E24&lt;&gt;0) * ('TẤT CẢ'!E7:E24&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D7" s="40" t="e" cm="1" vm="2">
+      <c r="D7" s="37" t="e" cm="1" vm="2">
         <f t="array" ref="D7">_xlfn._xlws.FILTER('TẤT CẢ'!D7:D24, ('TẤT CẢ'!E7:E24&lt;&gt;0) * ('TẤT CẢ'!E7:E24&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E7" s="40" t="e" cm="1" vm="2">
+      <c r="E7" s="37" t="e" cm="1" vm="2">
         <f t="array" ref="E7">_xlfn._xlws.FILTER('TẤT CẢ'!E7:E24, ('TẤT CẢ'!E7:E24&lt;&gt;0) * ('TẤT CẢ'!E7:E24&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F7" s="40" t="e" cm="1" vm="2">
+      <c r="F7" s="37" t="e" cm="1" vm="2">
         <f t="array" ref="F7">_xlfn._xlws.FILTER('TẤT CẢ'!F7:F24, ('TẤT CẢ'!E7:E24&lt;&gt;0) * ('TẤT CẢ'!E7:E24&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="39">
+      <c r="A8" s="36">
         <v>2</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="39">
+      <c r="A9" s="36">
         <v>3</v>
       </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
     </row>
     <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="39">
+      <c r="A10" s="36">
         <v>4</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
     </row>
     <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A11" s="39">
+      <c r="A11" s="36">
         <v>5</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
     </row>
     <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="39">
+      <c r="A12" s="36">
         <v>6</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
     </row>
     <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="39">
+      <c r="A13" s="36">
         <v>7</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="51"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
     </row>
     <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="39">
+      <c r="A14" s="36">
         <v>8</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
     </row>
     <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="39">
+      <c r="A15" s="36">
         <v>9</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="39"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
     </row>
     <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A16" s="39">
+      <c r="A16" s="36">
         <v>10</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
     </row>
     <row r="17" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="39">
+      <c r="A17" s="36">
         <v>11</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
     </row>
     <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="39">
+      <c r="A18" s="36">
         <v>12</v>
       </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="51"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
     </row>
     <row r="19" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A19" s="39">
+      <c r="A19" s="36">
         <v>13</v>
       </c>
-      <c r="B19" s="40"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="51"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
     </row>
     <row r="20" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A20" s="39">
+      <c r="A20" s="36">
         <v>14</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
     </row>
     <row r="21" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="39">
+      <c r="A21" s="36">
         <v>15</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="42"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="39"/>
     </row>
     <row r="22" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="39">
+      <c r="A22" s="36">
         <v>16</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="42"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="39"/>
     </row>
     <row r="23" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="43">
+      <c r="A23" s="40">
         <v>17</v>
       </c>
-      <c r="B23" s="87" t="s">
+      <c r="B23" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="88"/>
-      <c r="D23" s="89"/>
-      <c r="E23" s="44" t="e" vm="1">
+      <c r="C23" s="80"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="41" t="e" vm="1">
         <f>SUM(E7:E22)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F23" s="45"/>
+      <c r="F23" s="42"/>
     </row>
     <row r="27" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="F27" s="33" t="s">
+      <c r="F27" s="30" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2521,42 +2501,42 @@
   <sheetData>
     <row r="1" spans="1:14" ht="29.4" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
-      <c r="B1" s="77" t="s">
+      <c r="B1" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
     </row>
     <row r="2" spans="1:14" ht="24.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="72" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="79"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
-      <c r="D3" s="12"/>
+      <c r="D3" s="10"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -2565,1372 +2545,1372 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="24" t="s">
         <v>57</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="D4" s="12"/>
+      <c r="D4" s="10"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="L4" s="55" t="s">
+      <c r="L4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="M4" s="72">
+      <c r="M4" s="65">
         <f ca="1">NOW()</f>
-        <v>46287.616093055556</v>
+        <v>46297.399875578703</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="69" t="s">
+      <c r="B5" s="51"/>
+      <c r="C5" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
       <c r="L5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M5" s="14"/>
+      <c r="M5" s="12"/>
     </row>
     <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54"/>
-      <c r="B6" s="59" t="s">
+      <c r="A6" s="51"/>
+      <c r="B6" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="60" t="s">
+      <c r="C6" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="84"/>
-      <c r="E6" s="85"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="59" t="s">
+      <c r="D6" s="76"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="H6" s="60" t="s">
+      <c r="H6" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="84"/>
-      <c r="J6" s="85"/>
-      <c r="L6" s="25" t="s">
+      <c r="I6" s="76"/>
+      <c r="J6" s="77"/>
+      <c r="L6" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="M6" s="53">
+      <c r="M6" s="50">
         <f>I80+I83+C89</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="54"/>
-      <c r="B7" s="59" t="s">
+      <c r="A7" s="51"/>
+      <c r="B7" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="60" t="s">
+      <c r="C7" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="59" t="s">
+      <c r="D7" s="92"/>
+      <c r="E7" s="92"/>
+      <c r="F7" s="51"/>
+      <c r="G7" s="56" t="s">
         <v>64</v>
       </c>
-      <c r="H7" s="60" t="s">
+      <c r="H7" s="57" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="84"/>
-      <c r="J7" s="85"/>
-      <c r="L7" s="25" t="s">
+      <c r="I7" s="76"/>
+      <c r="J7" s="77"/>
+      <c r="L7" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="M7" s="28" t="e">
+      <c r="M7" s="25" t="e">
         <f>1-(M5/M6)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
-      <c r="B8" s="59" t="s">
+      <c r="A8" s="51"/>
+      <c r="B8" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="86"/>
-      <c r="E8" s="86"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="59" t="s">
+      <c r="C8" s="57"/>
+      <c r="D8" s="78"/>
+      <c r="E8" s="78"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="H8" s="60"/>
-      <c r="I8" s="86"/>
-      <c r="J8" s="86"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="78"/>
+      <c r="J8" s="78"/>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="54"/>
-      <c r="B9" s="59" t="s">
+      <c r="A9" s="51"/>
+      <c r="B9" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="60"/>
-      <c r="D9" s="86"/>
-      <c r="E9" s="86"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="59" t="s">
+      <c r="C9" s="57"/>
+      <c r="D9" s="78"/>
+      <c r="E9" s="78"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="60"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="78"/>
     </row>
     <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="58" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="56"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="55"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="52"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
-      <c r="L11" s="25"/>
+      <c r="L11" s="22"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="80" t="s">
+      <c r="A12" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="82" t="s">
+      <c r="B12" s="74" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="83"/>
-      <c r="E12" s="83"/>
-      <c r="F12" s="83"/>
-      <c r="G12" s="83"/>
-      <c r="H12" s="83"/>
-      <c r="I12" s="83"/>
-      <c r="J12" s="83"/>
-      <c r="K12" s="83"/>
-      <c r="L12" s="83"/>
-      <c r="M12" s="83"/>
-      <c r="N12" s="76" t="s">
+      <c r="C12" s="75"/>
+      <c r="D12" s="75"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="75"/>
+      <c r="G12" s="75"/>
+      <c r="H12" s="75"/>
+      <c r="I12" s="75"/>
+      <c r="J12" s="75"/>
+      <c r="K12" s="75"/>
+      <c r="L12" s="75"/>
+      <c r="M12" s="75"/>
+      <c r="N12" s="69" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="81"/>
-      <c r="B13" s="82" t="s">
+      <c r="A13" s="85"/>
+      <c r="B13" s="86" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="83"/>
-      <c r="I13" s="83"/>
-      <c r="J13" s="83"/>
-      <c r="K13" s="83"/>
-      <c r="L13" s="83"/>
-      <c r="M13" s="83"/>
-      <c r="N13" s="76"/>
+      <c r="C13" s="87"/>
+      <c r="D13" s="87"/>
+      <c r="E13" s="87"/>
+      <c r="F13" s="87"/>
+      <c r="G13" s="87"/>
+      <c r="H13" s="87"/>
+      <c r="I13" s="87"/>
+      <c r="J13" s="87"/>
+      <c r="K13" s="87"/>
+      <c r="L13" s="87"/>
+      <c r="M13" s="87"/>
+      <c r="N13" s="88"/>
     </row>
     <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65"/>
-      <c r="B14" s="66"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="64">
+      <c r="A14" s="61"/>
+      <c r="B14" s="89"/>
+      <c r="C14" s="89"/>
+      <c r="D14" s="89"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="89"/>
+      <c r="G14" s="89"/>
+      <c r="H14" s="89"/>
+      <c r="I14" s="89"/>
+      <c r="J14" s="89"/>
+      <c r="K14" s="89"/>
+      <c r="L14" s="89"/>
+      <c r="M14" s="90">
         <f>SUM(B14:L14)</f>
         <v>0</v>
       </c>
-      <c r="N14" s="54"/>
+      <c r="N14" s="61"/>
     </row>
     <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="65"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="64">
+      <c r="A15" s="61"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="89"/>
+      <c r="D15" s="89"/>
+      <c r="E15" s="89"/>
+      <c r="F15" s="89"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="89"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="90">
         <f t="shared" ref="M15:M75" si="0">SUM(B15:L15)</f>
         <v>0</v>
       </c>
-      <c r="N15" s="54"/>
+      <c r="N15" s="61"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="68"/>
-      <c r="B16" s="66"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="64">
+      <c r="A16" s="62"/>
+      <c r="B16" s="89"/>
+      <c r="C16" s="89"/>
+      <c r="D16" s="89"/>
+      <c r="E16" s="89"/>
+      <c r="F16" s="89"/>
+      <c r="G16" s="89"/>
+      <c r="H16" s="89"/>
+      <c r="I16" s="89"/>
+      <c r="J16" s="89"/>
+      <c r="K16" s="89"/>
+      <c r="L16" s="89"/>
+      <c r="M16" s="90">
         <f>SUM(B16:L16)</f>
         <v>0</v>
       </c>
-      <c r="N16" s="65"/>
+      <c r="N16" s="61"/>
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="54"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="64">
+      <c r="A17" s="61"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="89"/>
+      <c r="D17" s="89"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
+      <c r="K17" s="89"/>
+      <c r="L17" s="89"/>
+      <c r="M17" s="90">
         <f>SUM(B17:L17)</f>
         <v>0</v>
       </c>
-      <c r="N17" s="65"/>
+      <c r="N17" s="61"/>
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="54"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="64">
+      <c r="A18" s="61"/>
+      <c r="B18" s="89"/>
+      <c r="C18" s="89"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
+      <c r="G18" s="89"/>
+      <c r="H18" s="89"/>
+      <c r="I18" s="89"/>
+      <c r="J18" s="89"/>
+      <c r="K18" s="89"/>
+      <c r="L18" s="89"/>
+      <c r="M18" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N18" s="65"/>
+      <c r="N18" s="61"/>
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="24"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="64">
+      <c r="A19" s="62"/>
+      <c r="B19" s="89"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="89"/>
+      <c r="G19" s="89"/>
+      <c r="H19" s="89"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="89"/>
+      <c r="M19" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N19" s="65"/>
+      <c r="N19" s="61"/>
     </row>
     <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="67"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="64">
+      <c r="A20" s="62"/>
+      <c r="B20" s="89"/>
+      <c r="C20" s="89"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="89"/>
+      <c r="G20" s="89"/>
+      <c r="H20" s="89"/>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="89"/>
+      <c r="L20" s="89"/>
+      <c r="M20" s="90">
         <f>SUM(B20:L20)</f>
         <v>0</v>
       </c>
-      <c r="N20" s="65"/>
+      <c r="N20" s="61"/>
     </row>
     <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="65"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="64">
+      <c r="A21" s="61"/>
+      <c r="B21" s="89"/>
+      <c r="C21" s="89"/>
+      <c r="D21" s="89"/>
+      <c r="E21" s="89"/>
+      <c r="F21" s="89"/>
+      <c r="G21" s="89"/>
+      <c r="H21" s="89"/>
+      <c r="I21" s="89"/>
+      <c r="J21" s="89"/>
+      <c r="K21" s="89"/>
+      <c r="L21" s="89"/>
+      <c r="M21" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N21" s="65"/>
+      <c r="N21" s="61"/>
     </row>
     <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="24"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="64">
+      <c r="A22" s="62"/>
+      <c r="B22" s="89"/>
+      <c r="C22" s="89"/>
+      <c r="D22" s="89"/>
+      <c r="E22" s="89"/>
+      <c r="F22" s="89"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="89"/>
+      <c r="I22" s="89"/>
+      <c r="J22" s="89"/>
+      <c r="K22" s="89"/>
+      <c r="L22" s="89"/>
+      <c r="M22" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N22" s="65"/>
+      <c r="N22" s="61"/>
     </row>
     <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="24"/>
-      <c r="B23" s="54"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="64">
+      <c r="A23" s="62"/>
+      <c r="B23" s="61"/>
+      <c r="C23" s="89"/>
+      <c r="D23" s="89"/>
+      <c r="E23" s="89"/>
+      <c r="F23" s="89"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="89"/>
+      <c r="I23" s="89"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="89"/>
+      <c r="L23" s="89"/>
+      <c r="M23" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N23" s="65"/>
+      <c r="N23" s="61"/>
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="54"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="54"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="64">
+      <c r="A24" s="61"/>
+      <c r="B24" s="89"/>
+      <c r="C24" s="89"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="89"/>
+      <c r="F24" s="89"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="89"/>
+      <c r="I24" s="89"/>
+      <c r="J24" s="89"/>
+      <c r="K24" s="61"/>
+      <c r="L24" s="89"/>
+      <c r="M24" s="90">
         <f>SUM(B24:L24)</f>
         <v>0</v>
       </c>
-      <c r="N24" s="54"/>
+      <c r="N24" s="61"/>
     </row>
     <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="24"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="64">
+      <c r="A25" s="62"/>
+      <c r="B25" s="89"/>
+      <c r="C25" s="89"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="89"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="89"/>
+      <c r="H25" s="89"/>
+      <c r="I25" s="89"/>
+      <c r="J25" s="89"/>
+      <c r="K25" s="89"/>
+      <c r="L25" s="89"/>
+      <c r="M25" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N25" s="54"/>
+      <c r="N25" s="61"/>
     </row>
     <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="54"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="64">
+      <c r="A26" s="61"/>
+      <c r="B26" s="89"/>
+      <c r="C26" s="89"/>
+      <c r="D26" s="89"/>
+      <c r="E26" s="89"/>
+      <c r="F26" s="89"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
+      <c r="I26" s="89"/>
+      <c r="J26" s="89"/>
+      <c r="K26" s="89"/>
+      <c r="L26" s="89"/>
+      <c r="M26" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N26" s="65"/>
+      <c r="N26" s="61"/>
     </row>
     <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="24"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="64">
+      <c r="A27" s="62"/>
+      <c r="B27" s="89"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="89"/>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="89"/>
+      <c r="J27" s="89"/>
+      <c r="K27" s="89"/>
+      <c r="L27" s="89"/>
+      <c r="M27" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N27" s="54"/>
+      <c r="N27" s="61"/>
     </row>
     <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="54"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="64">
+      <c r="A28" s="61"/>
+      <c r="B28" s="89"/>
+      <c r="C28" s="89"/>
+      <c r="D28" s="89"/>
+      <c r="E28" s="89"/>
+      <c r="F28" s="89"/>
+      <c r="G28" s="89"/>
+      <c r="H28" s="89"/>
+      <c r="I28" s="89"/>
+      <c r="J28" s="89"/>
+      <c r="K28" s="89"/>
+      <c r="L28" s="89"/>
+      <c r="M28" s="90">
         <f>SUM(B28:L28)</f>
         <v>0</v>
       </c>
-      <c r="N28" s="54"/>
+      <c r="N28" s="61"/>
     </row>
     <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="24"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="64">
+      <c r="A29" s="62"/>
+      <c r="B29" s="89"/>
+      <c r="C29" s="89"/>
+      <c r="D29" s="89"/>
+      <c r="E29" s="89"/>
+      <c r="F29" s="89"/>
+      <c r="G29" s="89"/>
+      <c r="H29" s="89"/>
+      <c r="I29" s="89"/>
+      <c r="J29" s="89"/>
+      <c r="K29" s="89"/>
+      <c r="L29" s="89"/>
+      <c r="M29" s="90">
         <f>SUM(B29:L29)</f>
         <v>0</v>
       </c>
-      <c r="N29" s="65"/>
+      <c r="N29" s="61"/>
     </row>
     <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="24"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="64">
+      <c r="A30" s="62"/>
+      <c r="B30" s="89"/>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
+      <c r="E30" s="89"/>
+      <c r="F30" s="89"/>
+      <c r="G30" s="89"/>
+      <c r="H30" s="89"/>
+      <c r="I30" s="89"/>
+      <c r="J30" s="89"/>
+      <c r="K30" s="89"/>
+      <c r="L30" s="89"/>
+      <c r="M30" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N30" s="65"/>
+      <c r="N30" s="61"/>
     </row>
     <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="64">
+      <c r="A31" s="91"/>
+      <c r="B31" s="61"/>
+      <c r="C31" s="89"/>
+      <c r="D31" s="89"/>
+      <c r="E31" s="89"/>
+      <c r="F31" s="89"/>
+      <c r="G31" s="89"/>
+      <c r="H31" s="89"/>
+      <c r="I31" s="89"/>
+      <c r="J31" s="89"/>
+      <c r="K31" s="89"/>
+      <c r="L31" s="89"/>
+      <c r="M31" s="90">
         <f>SUM(B31:L31)</f>
         <v>0</v>
       </c>
-      <c r="N31" s="65"/>
+      <c r="N31" s="61"/>
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="54"/>
-      <c r="B32" s="24"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="64"/>
-      <c r="N32" s="54"/>
+      <c r="A32" s="61"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="89"/>
+      <c r="D32" s="89"/>
+      <c r="E32" s="89"/>
+      <c r="F32" s="89"/>
+      <c r="G32" s="89"/>
+      <c r="H32" s="89"/>
+      <c r="I32" s="89"/>
+      <c r="J32" s="89"/>
+      <c r="K32" s="89"/>
+      <c r="L32" s="89"/>
+      <c r="M32" s="90"/>
+      <c r="N32" s="61"/>
     </row>
     <row r="33" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="64">
+      <c r="A33" s="91"/>
+      <c r="B33" s="89"/>
+      <c r="C33" s="89"/>
+      <c r="D33" s="89"/>
+      <c r="E33" s="89"/>
+      <c r="F33" s="89"/>
+      <c r="G33" s="89"/>
+      <c r="H33" s="89"/>
+      <c r="I33" s="89"/>
+      <c r="J33" s="89"/>
+      <c r="K33" s="89"/>
+      <c r="L33" s="89"/>
+      <c r="M33" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N33" s="65"/>
+      <c r="N33" s="61"/>
     </row>
     <row r="34" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="11"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="64">
+      <c r="A34" s="91"/>
+      <c r="B34" s="89"/>
+      <c r="C34" s="89"/>
+      <c r="D34" s="89"/>
+      <c r="E34" s="89"/>
+      <c r="F34" s="91"/>
+      <c r="G34" s="89"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="89"/>
+      <c r="J34" s="89"/>
+      <c r="K34" s="89"/>
+      <c r="L34" s="89"/>
+      <c r="M34" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N34" s="65"/>
+      <c r="N34" s="61"/>
     </row>
     <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="54"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-      <c r="M35" s="64">
+      <c r="A35" s="61"/>
+      <c r="B35" s="89"/>
+      <c r="C35" s="89"/>
+      <c r="D35" s="89"/>
+      <c r="E35" s="89"/>
+      <c r="F35" s="89"/>
+      <c r="G35" s="89"/>
+      <c r="H35" s="89"/>
+      <c r="I35" s="89"/>
+      <c r="J35" s="89"/>
+      <c r="K35" s="89"/>
+      <c r="L35" s="89"/>
+      <c r="M35" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N35" s="65"/>
+      <c r="N35" s="61"/>
     </row>
     <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="54"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
-      <c r="M36" s="64">
+      <c r="A36" s="61"/>
+      <c r="B36" s="89"/>
+      <c r="C36" s="89"/>
+      <c r="D36" s="89"/>
+      <c r="E36" s="89"/>
+      <c r="F36" s="89"/>
+      <c r="G36" s="89"/>
+      <c r="H36" s="89"/>
+      <c r="I36" s="89"/>
+      <c r="J36" s="89"/>
+      <c r="K36" s="89"/>
+      <c r="L36" s="89"/>
+      <c r="M36" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N36" s="65"/>
+      <c r="N36" s="61"/>
     </row>
     <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="11"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
-      <c r="J37" s="10"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="64">
+      <c r="A37" s="91"/>
+      <c r="B37" s="89"/>
+      <c r="C37" s="89"/>
+      <c r="D37" s="89"/>
+      <c r="E37" s="89"/>
+      <c r="F37" s="89"/>
+      <c r="G37" s="89"/>
+      <c r="H37" s="89"/>
+      <c r="I37" s="89"/>
+      <c r="J37" s="89"/>
+      <c r="K37" s="89"/>
+      <c r="L37" s="89"/>
+      <c r="M37" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N37" s="65"/>
+      <c r="N37" s="61"/>
     </row>
     <row r="38" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="11"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="64">
+      <c r="A38" s="91"/>
+      <c r="B38" s="89"/>
+      <c r="C38" s="89"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="89"/>
+      <c r="F38" s="89"/>
+      <c r="G38" s="89"/>
+      <c r="H38" s="89"/>
+      <c r="I38" s="89"/>
+      <c r="J38" s="89"/>
+      <c r="K38" s="89"/>
+      <c r="L38" s="89"/>
+      <c r="M38" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N38" s="65"/>
+      <c r="N38" s="61"/>
     </row>
     <row r="39" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="11"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="10"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
-      <c r="M39" s="64">
+      <c r="A39" s="91"/>
+      <c r="B39" s="89"/>
+      <c r="C39" s="89"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="89"/>
+      <c r="F39" s="89"/>
+      <c r="G39" s="89"/>
+      <c r="H39" s="89"/>
+      <c r="I39" s="89"/>
+      <c r="J39" s="89"/>
+      <c r="K39" s="89"/>
+      <c r="L39" s="89"/>
+      <c r="M39" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N39" s="65"/>
+      <c r="N39" s="61"/>
     </row>
     <row r="40" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="11"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="10"/>
-      <c r="J40" s="10"/>
-      <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="64">
+      <c r="A40" s="91"/>
+      <c r="B40" s="89"/>
+      <c r="C40" s="89"/>
+      <c r="D40" s="89"/>
+      <c r="E40" s="89"/>
+      <c r="F40" s="89"/>
+      <c r="G40" s="89"/>
+      <c r="H40" s="89"/>
+      <c r="I40" s="89"/>
+      <c r="J40" s="89"/>
+      <c r="K40" s="89"/>
+      <c r="L40" s="89"/>
+      <c r="M40" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N40" s="65"/>
+      <c r="N40" s="61"/>
     </row>
     <row r="41" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="11"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10"/>
-      <c r="K41" s="10"/>
-      <c r="L41" s="10"/>
-      <c r="M41" s="64">
+      <c r="A41" s="91"/>
+      <c r="B41" s="89"/>
+      <c r="C41" s="89"/>
+      <c r="D41" s="89"/>
+      <c r="E41" s="89"/>
+      <c r="F41" s="89"/>
+      <c r="G41" s="89"/>
+      <c r="H41" s="89"/>
+      <c r="I41" s="89"/>
+      <c r="J41" s="89"/>
+      <c r="K41" s="89"/>
+      <c r="L41" s="89"/>
+      <c r="M41" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N41" s="65"/>
+      <c r="N41" s="61"/>
     </row>
     <row r="42" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="11"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="64">
+      <c r="A42" s="91"/>
+      <c r="B42" s="89"/>
+      <c r="C42" s="89"/>
+      <c r="D42" s="89"/>
+      <c r="E42" s="89"/>
+      <c r="F42" s="89"/>
+      <c r="G42" s="89"/>
+      <c r="H42" s="89"/>
+      <c r="I42" s="89"/>
+      <c r="J42" s="89"/>
+      <c r="K42" s="89"/>
+      <c r="L42" s="89"/>
+      <c r="M42" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N42" s="54"/>
+      <c r="N42" s="61"/>
     </row>
     <row r="43" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="11"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="10"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
-      <c r="L43" s="10"/>
-      <c r="M43" s="64">
+      <c r="A43" s="91"/>
+      <c r="B43" s="89"/>
+      <c r="C43" s="89"/>
+      <c r="D43" s="89"/>
+      <c r="E43" s="89"/>
+      <c r="F43" s="89"/>
+      <c r="G43" s="89"/>
+      <c r="H43" s="89"/>
+      <c r="I43" s="89"/>
+      <c r="J43" s="89"/>
+      <c r="K43" s="89"/>
+      <c r="L43" s="89"/>
+      <c r="M43" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N43" s="65"/>
+      <c r="N43" s="61"/>
     </row>
     <row r="44" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="11"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="64">
+      <c r="A44" s="91"/>
+      <c r="B44" s="89"/>
+      <c r="C44" s="89"/>
+      <c r="D44" s="89"/>
+      <c r="E44" s="89"/>
+      <c r="F44" s="89"/>
+      <c r="G44" s="89"/>
+      <c r="H44" s="89"/>
+      <c r="I44" s="89"/>
+      <c r="J44" s="89"/>
+      <c r="K44" s="89"/>
+      <c r="L44" s="89"/>
+      <c r="M44" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N44" s="54"/>
+      <c r="N44" s="61"/>
     </row>
     <row r="45" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="54"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="10"/>
-      <c r="G45" s="10"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="10"/>
-      <c r="J45" s="10"/>
-      <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="64">
+      <c r="A45" s="61"/>
+      <c r="B45" s="89"/>
+      <c r="C45" s="89"/>
+      <c r="D45" s="89"/>
+      <c r="E45" s="89"/>
+      <c r="F45" s="89"/>
+      <c r="G45" s="89"/>
+      <c r="H45" s="89"/>
+      <c r="I45" s="89"/>
+      <c r="J45" s="89"/>
+      <c r="K45" s="89"/>
+      <c r="L45" s="89"/>
+      <c r="M45" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N45" s="65"/>
+      <c r="N45" s="61"/>
     </row>
     <row r="46" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="11"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
-      <c r="K46" s="10"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="64">
+      <c r="A46" s="91"/>
+      <c r="B46" s="89"/>
+      <c r="C46" s="89"/>
+      <c r="D46" s="89"/>
+      <c r="E46" s="89"/>
+      <c r="F46" s="89"/>
+      <c r="G46" s="89"/>
+      <c r="H46" s="89"/>
+      <c r="I46" s="89"/>
+      <c r="J46" s="89"/>
+      <c r="K46" s="89"/>
+      <c r="L46" s="89"/>
+      <c r="M46" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N46" s="65"/>
+      <c r="N46" s="61"/>
     </row>
     <row r="47" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="11"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="10"/>
-      <c r="K47" s="10"/>
-      <c r="L47" s="10"/>
-      <c r="M47" s="64">
+      <c r="A47" s="91"/>
+      <c r="B47" s="89"/>
+      <c r="C47" s="89"/>
+      <c r="D47" s="89"/>
+      <c r="E47" s="89"/>
+      <c r="F47" s="89"/>
+      <c r="G47" s="89"/>
+      <c r="H47" s="89"/>
+      <c r="I47" s="89"/>
+      <c r="J47" s="89"/>
+      <c r="K47" s="89"/>
+      <c r="L47" s="89"/>
+      <c r="M47" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N47" s="65"/>
+      <c r="N47" s="61"/>
     </row>
     <row r="48" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="11"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="10"/>
-      <c r="K48" s="10"/>
-      <c r="L48" s="10"/>
-      <c r="M48" s="64">
+      <c r="A48" s="91"/>
+      <c r="B48" s="89"/>
+      <c r="C48" s="89"/>
+      <c r="D48" s="89"/>
+      <c r="E48" s="89"/>
+      <c r="F48" s="89"/>
+      <c r="G48" s="89"/>
+      <c r="H48" s="89"/>
+      <c r="I48" s="89"/>
+      <c r="J48" s="89"/>
+      <c r="K48" s="89"/>
+      <c r="L48" s="89"/>
+      <c r="M48" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N48" s="70"/>
+      <c r="N48" s="64"/>
     </row>
     <row r="49" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="11"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
-      <c r="I49" s="10"/>
-      <c r="J49" s="10"/>
-      <c r="K49" s="10"/>
-      <c r="L49" s="10"/>
-      <c r="M49" s="64">
+      <c r="A49" s="91"/>
+      <c r="B49" s="89"/>
+      <c r="C49" s="89"/>
+      <c r="D49" s="89"/>
+      <c r="E49" s="89"/>
+      <c r="F49" s="89"/>
+      <c r="G49" s="89"/>
+      <c r="H49" s="89"/>
+      <c r="I49" s="89"/>
+      <c r="J49" s="89"/>
+      <c r="K49" s="89"/>
+      <c r="L49" s="89"/>
+      <c r="M49" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N49" s="65"/>
+      <c r="N49" s="61"/>
     </row>
     <row r="50" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="11"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="10"/>
-      <c r="K50" s="10"/>
-      <c r="L50" s="10"/>
-      <c r="M50" s="64">
+      <c r="A50" s="91"/>
+      <c r="B50" s="89"/>
+      <c r="C50" s="89"/>
+      <c r="D50" s="89"/>
+      <c r="E50" s="89"/>
+      <c r="F50" s="89"/>
+      <c r="G50" s="89"/>
+      <c r="H50" s="89"/>
+      <c r="I50" s="89"/>
+      <c r="J50" s="89"/>
+      <c r="K50" s="89"/>
+      <c r="L50" s="89"/>
+      <c r="M50" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N50" s="65"/>
+      <c r="N50" s="61"/>
     </row>
     <row r="51" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="11"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-      <c r="J51" s="10"/>
-      <c r="K51" s="10"/>
-      <c r="L51" s="10"/>
-      <c r="M51" s="64">
+      <c r="A51" s="91"/>
+      <c r="B51" s="89"/>
+      <c r="C51" s="89"/>
+      <c r="D51" s="89"/>
+      <c r="E51" s="89"/>
+      <c r="F51" s="89"/>
+      <c r="G51" s="89"/>
+      <c r="H51" s="89"/>
+      <c r="I51" s="89"/>
+      <c r="J51" s="89"/>
+      <c r="K51" s="89"/>
+      <c r="L51" s="89"/>
+      <c r="M51" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N51" s="54"/>
+      <c r="N51" s="61"/>
     </row>
     <row r="52" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="11"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="64">
+      <c r="A52" s="91"/>
+      <c r="B52" s="89"/>
+      <c r="C52" s="89"/>
+      <c r="D52" s="89"/>
+      <c r="E52" s="89"/>
+      <c r="F52" s="89"/>
+      <c r="G52" s="89"/>
+      <c r="H52" s="89"/>
+      <c r="I52" s="89"/>
+      <c r="J52" s="89"/>
+      <c r="K52" s="89"/>
+      <c r="L52" s="89"/>
+      <c r="M52" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N52" s="54"/>
+      <c r="N52" s="61"/>
     </row>
     <row r="53" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="11"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
-      <c r="H53" s="10"/>
-      <c r="I53" s="10"/>
-      <c r="J53" s="10"/>
-      <c r="K53" s="10"/>
-      <c r="L53" s="10"/>
-      <c r="M53" s="64">
+      <c r="A53" s="91"/>
+      <c r="B53" s="89"/>
+      <c r="C53" s="89"/>
+      <c r="D53" s="89"/>
+      <c r="E53" s="89"/>
+      <c r="F53" s="89"/>
+      <c r="G53" s="89"/>
+      <c r="H53" s="89"/>
+      <c r="I53" s="89"/>
+      <c r="J53" s="89"/>
+      <c r="K53" s="89"/>
+      <c r="L53" s="89"/>
+      <c r="M53" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N53" s="54"/>
+      <c r="N53" s="61"/>
     </row>
     <row r="54" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="11"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
-      <c r="M54" s="64">
+      <c r="A54" s="91"/>
+      <c r="B54" s="89"/>
+      <c r="C54" s="89"/>
+      <c r="D54" s="89"/>
+      <c r="E54" s="89"/>
+      <c r="F54" s="89"/>
+      <c r="G54" s="89"/>
+      <c r="H54" s="89"/>
+      <c r="I54" s="89"/>
+      <c r="J54" s="89"/>
+      <c r="K54" s="89"/>
+      <c r="L54" s="89"/>
+      <c r="M54" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N54" s="65"/>
+      <c r="N54" s="61"/>
     </row>
     <row r="55" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="11"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="10"/>
-      <c r="J55" s="10"/>
-      <c r="K55" s="10"/>
-      <c r="L55" s="10"/>
-      <c r="M55" s="64">
+      <c r="A55" s="91"/>
+      <c r="B55" s="89"/>
+      <c r="C55" s="89"/>
+      <c r="D55" s="89"/>
+      <c r="E55" s="89"/>
+      <c r="F55" s="89"/>
+      <c r="G55" s="89"/>
+      <c r="H55" s="89"/>
+      <c r="I55" s="89"/>
+      <c r="J55" s="89"/>
+      <c r="K55" s="89"/>
+      <c r="L55" s="89"/>
+      <c r="M55" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N55" s="65"/>
+      <c r="N55" s="61"/>
     </row>
     <row r="56" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="11"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
-      <c r="H56" s="10"/>
-      <c r="I56" s="10"/>
-      <c r="J56" s="10"/>
-      <c r="K56" s="10"/>
-      <c r="L56" s="10"/>
-      <c r="M56" s="64">
+      <c r="A56" s="91"/>
+      <c r="B56" s="89"/>
+      <c r="C56" s="89"/>
+      <c r="D56" s="89"/>
+      <c r="E56" s="89"/>
+      <c r="F56" s="89"/>
+      <c r="G56" s="89"/>
+      <c r="H56" s="89"/>
+      <c r="I56" s="89"/>
+      <c r="J56" s="89"/>
+      <c r="K56" s="89"/>
+      <c r="L56" s="89"/>
+      <c r="M56" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N56" s="65"/>
+      <c r="N56" s="61"/>
     </row>
     <row r="57" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="11"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="10"/>
-      <c r="H57" s="10"/>
-      <c r="I57" s="10"/>
-      <c r="J57" s="10"/>
-      <c r="K57" s="10"/>
-      <c r="L57" s="10"/>
-      <c r="M57" s="64">
+      <c r="A57" s="91"/>
+      <c r="B57" s="89"/>
+      <c r="C57" s="89"/>
+      <c r="D57" s="89"/>
+      <c r="E57" s="89"/>
+      <c r="F57" s="89"/>
+      <c r="G57" s="89"/>
+      <c r="H57" s="89"/>
+      <c r="I57" s="89"/>
+      <c r="J57" s="89"/>
+      <c r="K57" s="89"/>
+      <c r="L57" s="89"/>
+      <c r="M57" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N57" s="65"/>
+      <c r="N57" s="61"/>
     </row>
     <row r="58" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="11"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
-      <c r="K58" s="10"/>
-      <c r="L58" s="10"/>
-      <c r="M58" s="64">
+      <c r="A58" s="91"/>
+      <c r="B58" s="89"/>
+      <c r="C58" s="89"/>
+      <c r="D58" s="89"/>
+      <c r="E58" s="89"/>
+      <c r="F58" s="89"/>
+      <c r="G58" s="89"/>
+      <c r="H58" s="89"/>
+      <c r="I58" s="89"/>
+      <c r="J58" s="89"/>
+      <c r="K58" s="89"/>
+      <c r="L58" s="89"/>
+      <c r="M58" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N58" s="65"/>
+      <c r="N58" s="61"/>
     </row>
     <row r="59" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="11"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
-      <c r="H59" s="10"/>
-      <c r="I59" s="10"/>
-      <c r="J59" s="10"/>
-      <c r="K59" s="10"/>
-      <c r="L59" s="10"/>
-      <c r="M59" s="64">
+      <c r="A59" s="91"/>
+      <c r="B59" s="89"/>
+      <c r="C59" s="89"/>
+      <c r="D59" s="89"/>
+      <c r="E59" s="89"/>
+      <c r="F59" s="89"/>
+      <c r="G59" s="89"/>
+      <c r="H59" s="89"/>
+      <c r="I59" s="89"/>
+      <c r="J59" s="89"/>
+      <c r="K59" s="89"/>
+      <c r="L59" s="89"/>
+      <c r="M59" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N59" s="65"/>
+      <c r="N59" s="61"/>
     </row>
     <row r="60" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="11"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
-      <c r="K60" s="10"/>
-      <c r="L60" s="10"/>
-      <c r="M60" s="64">
+      <c r="A60" s="91"/>
+      <c r="B60" s="89"/>
+      <c r="C60" s="89"/>
+      <c r="D60" s="89"/>
+      <c r="E60" s="89"/>
+      <c r="F60" s="89"/>
+      <c r="G60" s="89"/>
+      <c r="H60" s="89"/>
+      <c r="I60" s="89"/>
+      <c r="J60" s="89"/>
+      <c r="K60" s="89"/>
+      <c r="L60" s="89"/>
+      <c r="M60" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N60" s="54"/>
+      <c r="N60" s="61"/>
     </row>
     <row r="61" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="11"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
-      <c r="L61" s="10"/>
-      <c r="M61" s="64">
+      <c r="A61" s="91"/>
+      <c r="B61" s="89"/>
+      <c r="C61" s="89"/>
+      <c r="D61" s="89"/>
+      <c r="E61" s="89"/>
+      <c r="F61" s="89"/>
+      <c r="G61" s="89"/>
+      <c r="H61" s="89"/>
+      <c r="I61" s="89"/>
+      <c r="J61" s="89"/>
+      <c r="K61" s="89"/>
+      <c r="L61" s="89"/>
+      <c r="M61" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N61" s="65"/>
+      <c r="N61" s="61"/>
     </row>
     <row r="62" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="11"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
-      <c r="I62" s="10"/>
-      <c r="J62" s="10"/>
-      <c r="K62" s="10"/>
-      <c r="L62" s="10"/>
-      <c r="M62" s="64">
+      <c r="A62" s="91"/>
+      <c r="B62" s="89"/>
+      <c r="C62" s="89"/>
+      <c r="D62" s="89"/>
+      <c r="E62" s="89"/>
+      <c r="F62" s="89"/>
+      <c r="G62" s="89"/>
+      <c r="H62" s="89"/>
+      <c r="I62" s="89"/>
+      <c r="J62" s="89"/>
+      <c r="K62" s="89"/>
+      <c r="L62" s="89"/>
+      <c r="M62" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N62" s="65"/>
+      <c r="N62" s="61"/>
     </row>
     <row r="63" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="11"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
-      <c r="M63" s="64">
+      <c r="A63" s="91"/>
+      <c r="B63" s="89"/>
+      <c r="C63" s="89"/>
+      <c r="D63" s="89"/>
+      <c r="E63" s="89"/>
+      <c r="F63" s="89"/>
+      <c r="G63" s="89"/>
+      <c r="H63" s="89"/>
+      <c r="I63" s="89"/>
+      <c r="J63" s="89"/>
+      <c r="K63" s="89"/>
+      <c r="L63" s="89"/>
+      <c r="M63" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N63" s="65"/>
+      <c r="N63" s="61"/>
     </row>
     <row r="64" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="11"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="10"/>
-      <c r="M64" s="64">
+      <c r="A64" s="91"/>
+      <c r="B64" s="89"/>
+      <c r="C64" s="89"/>
+      <c r="D64" s="89"/>
+      <c r="E64" s="89"/>
+      <c r="F64" s="89"/>
+      <c r="G64" s="89"/>
+      <c r="H64" s="89"/>
+      <c r="I64" s="89"/>
+      <c r="J64" s="89"/>
+      <c r="K64" s="89"/>
+      <c r="L64" s="89"/>
+      <c r="M64" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N64" s="65"/>
+      <c r="N64" s="61"/>
     </row>
     <row r="65" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="11"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="10"/>
-      <c r="H65" s="10"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="10"/>
-      <c r="K65" s="10"/>
-      <c r="L65" s="10"/>
-      <c r="M65" s="64">
+      <c r="A65" s="91"/>
+      <c r="B65" s="89"/>
+      <c r="C65" s="89"/>
+      <c r="D65" s="89"/>
+      <c r="E65" s="89"/>
+      <c r="F65" s="89"/>
+      <c r="G65" s="89"/>
+      <c r="H65" s="89"/>
+      <c r="I65" s="89"/>
+      <c r="J65" s="89"/>
+      <c r="K65" s="89"/>
+      <c r="L65" s="89"/>
+      <c r="M65" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N65" s="65"/>
+      <c r="N65" s="61"/>
     </row>
     <row r="66" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="11"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
-      <c r="E66" s="10"/>
-      <c r="F66" s="10"/>
-      <c r="G66" s="10"/>
-      <c r="H66" s="10"/>
-      <c r="I66" s="10"/>
-      <c r="J66" s="10"/>
-      <c r="K66" s="10"/>
-      <c r="L66" s="10"/>
-      <c r="M66" s="64">
+      <c r="A66" s="91"/>
+      <c r="B66" s="89"/>
+      <c r="C66" s="89"/>
+      <c r="D66" s="89"/>
+      <c r="E66" s="89"/>
+      <c r="F66" s="89"/>
+      <c r="G66" s="89"/>
+      <c r="H66" s="89"/>
+      <c r="I66" s="89"/>
+      <c r="J66" s="89"/>
+      <c r="K66" s="89"/>
+      <c r="L66" s="89"/>
+      <c r="M66" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N66" s="65"/>
+      <c r="N66" s="61"/>
     </row>
     <row r="67" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="11"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
-      <c r="F67" s="10"/>
-      <c r="G67" s="10"/>
-      <c r="H67" s="10"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
-      <c r="K67" s="10"/>
-      <c r="L67" s="10"/>
-      <c r="M67" s="64">
+      <c r="A67" s="91"/>
+      <c r="B67" s="89"/>
+      <c r="C67" s="89"/>
+      <c r="D67" s="89"/>
+      <c r="E67" s="89"/>
+      <c r="F67" s="89"/>
+      <c r="G67" s="89"/>
+      <c r="H67" s="89"/>
+      <c r="I67" s="89"/>
+      <c r="J67" s="89"/>
+      <c r="K67" s="89"/>
+      <c r="L67" s="89"/>
+      <c r="M67" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N67" s="65"/>
+      <c r="N67" s="61"/>
     </row>
     <row r="68" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="11"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
-      <c r="G68" s="10"/>
-      <c r="H68" s="10"/>
-      <c r="I68" s="10"/>
-      <c r="J68" s="10"/>
-      <c r="K68" s="10"/>
-      <c r="L68" s="10"/>
-      <c r="M68" s="64">
+      <c r="A68" s="91"/>
+      <c r="B68" s="89"/>
+      <c r="C68" s="89"/>
+      <c r="D68" s="89"/>
+      <c r="E68" s="89"/>
+      <c r="F68" s="89"/>
+      <c r="G68" s="89"/>
+      <c r="H68" s="89"/>
+      <c r="I68" s="89"/>
+      <c r="J68" s="89"/>
+      <c r="K68" s="89"/>
+      <c r="L68" s="89"/>
+      <c r="M68" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N68" s="65"/>
+      <c r="N68" s="61"/>
     </row>
     <row r="69" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="11"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
-      <c r="G69" s="10"/>
-      <c r="H69" s="10"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="10"/>
-      <c r="K69" s="10"/>
-      <c r="L69" s="10"/>
-      <c r="M69" s="64">
+      <c r="A69" s="91"/>
+      <c r="B69" s="89"/>
+      <c r="C69" s="89"/>
+      <c r="D69" s="89"/>
+      <c r="E69" s="89"/>
+      <c r="F69" s="89"/>
+      <c r="G69" s="89"/>
+      <c r="H69" s="89"/>
+      <c r="I69" s="89"/>
+      <c r="J69" s="89"/>
+      <c r="K69" s="89"/>
+      <c r="L69" s="89"/>
+      <c r="M69" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N69" s="65"/>
+      <c r="N69" s="61"/>
     </row>
     <row r="70" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="11"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="10"/>
-      <c r="K70" s="10"/>
-      <c r="L70" s="10"/>
-      <c r="M70" s="64">
+      <c r="A70" s="91"/>
+      <c r="B70" s="89"/>
+      <c r="C70" s="89"/>
+      <c r="D70" s="89"/>
+      <c r="E70" s="89"/>
+      <c r="F70" s="89"/>
+      <c r="G70" s="89"/>
+      <c r="H70" s="89"/>
+      <c r="I70" s="89"/>
+      <c r="J70" s="89"/>
+      <c r="K70" s="89"/>
+      <c r="L70" s="89"/>
+      <c r="M70" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N70" s="65"/>
+      <c r="N70" s="61"/>
     </row>
     <row r="71" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="11"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="10"/>
-      <c r="E71" s="10"/>
-      <c r="F71" s="10"/>
-      <c r="G71" s="10"/>
-      <c r="H71" s="10"/>
-      <c r="I71" s="10"/>
-      <c r="J71" s="10"/>
-      <c r="K71" s="10"/>
-      <c r="L71" s="10"/>
-      <c r="M71" s="64">
+      <c r="A71" s="91"/>
+      <c r="B71" s="89"/>
+      <c r="C71" s="89"/>
+      <c r="D71" s="89"/>
+      <c r="E71" s="89"/>
+      <c r="F71" s="89"/>
+      <c r="G71" s="89"/>
+      <c r="H71" s="89"/>
+      <c r="I71" s="89"/>
+      <c r="J71" s="89"/>
+      <c r="K71" s="89"/>
+      <c r="L71" s="89"/>
+      <c r="M71" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N71" s="65"/>
+      <c r="N71" s="61"/>
     </row>
     <row r="72" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="11"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
-      <c r="I72" s="10"/>
-      <c r="J72" s="10"/>
-      <c r="K72" s="10"/>
-      <c r="L72" s="10"/>
-      <c r="M72" s="64">
+      <c r="A72" s="91"/>
+      <c r="B72" s="89"/>
+      <c r="C72" s="89"/>
+      <c r="D72" s="89"/>
+      <c r="E72" s="89"/>
+      <c r="F72" s="89"/>
+      <c r="G72" s="89"/>
+      <c r="H72" s="89"/>
+      <c r="I72" s="89"/>
+      <c r="J72" s="89"/>
+      <c r="K72" s="89"/>
+      <c r="L72" s="89"/>
+      <c r="M72" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N72" s="65"/>
+      <c r="N72" s="61"/>
     </row>
     <row r="73" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="11"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="10"/>
-      <c r="E73" s="10"/>
-      <c r="F73" s="10"/>
-      <c r="G73" s="10"/>
-      <c r="H73" s="10"/>
-      <c r="I73" s="10"/>
-      <c r="J73" s="10"/>
-      <c r="K73" s="10"/>
-      <c r="L73" s="10"/>
-      <c r="M73" s="64">
+      <c r="A73" s="91"/>
+      <c r="B73" s="89"/>
+      <c r="C73" s="89"/>
+      <c r="D73" s="89"/>
+      <c r="E73" s="89"/>
+      <c r="F73" s="89"/>
+      <c r="G73" s="89"/>
+      <c r="H73" s="89"/>
+      <c r="I73" s="89"/>
+      <c r="J73" s="89"/>
+      <c r="K73" s="89"/>
+      <c r="L73" s="89"/>
+      <c r="M73" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N73" s="65"/>
+      <c r="N73" s="61"/>
     </row>
     <row r="74" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="11"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="10"/>
-      <c r="E74" s="10"/>
-      <c r="F74" s="10"/>
-      <c r="G74" s="10"/>
-      <c r="H74" s="10"/>
-      <c r="I74" s="10"/>
-      <c r="J74" s="10"/>
-      <c r="K74" s="10"/>
-      <c r="L74" s="10"/>
-      <c r="M74" s="64">
+      <c r="A74" s="91"/>
+      <c r="B74" s="89"/>
+      <c r="C74" s="89"/>
+      <c r="D74" s="89"/>
+      <c r="E74" s="89"/>
+      <c r="F74" s="89"/>
+      <c r="G74" s="89"/>
+      <c r="H74" s="89"/>
+      <c r="I74" s="89"/>
+      <c r="J74" s="89"/>
+      <c r="K74" s="89"/>
+      <c r="L74" s="89"/>
+      <c r="M74" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N74" s="65"/>
+      <c r="N74" s="61"/>
     </row>
     <row r="75" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="71"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="10"/>
-      <c r="E75" s="10"/>
-      <c r="F75" s="10"/>
-      <c r="G75" s="10"/>
-      <c r="H75" s="10"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="10"/>
-      <c r="K75" s="10"/>
-      <c r="L75" s="10"/>
-      <c r="M75" s="64">
+      <c r="A75" s="91"/>
+      <c r="B75" s="89"/>
+      <c r="C75" s="89"/>
+      <c r="D75" s="89"/>
+      <c r="E75" s="89"/>
+      <c r="F75" s="89"/>
+      <c r="G75" s="89"/>
+      <c r="H75" s="89"/>
+      <c r="I75" s="89"/>
+      <c r="J75" s="89"/>
+      <c r="K75" s="89"/>
+      <c r="L75" s="89"/>
+      <c r="M75" s="90">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="N75" s="65"/>
+      <c r="N75" s="61"/>
     </row>
     <row r="76" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="38"/>
+      <c r="A76" s="35"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
-      <c r="L76" s="62" t="s">
+      <c r="L76" s="59" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="26" t="s">
+      <c r="A77" s="23" t="s">
         <v>78</v>
       </c>
       <c r="B77" s="6"/>
@@ -3944,30 +3924,30 @@
       <c r="J77" s="2"/>
     </row>
     <row r="78" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="21" t="s">
+      <c r="A78" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="B78" s="29" t="s">
+      <c r="B78" s="26" t="s">
         <v>80</v>
       </c>
       <c r="C78" s="9">
         <f>SUMIF(A14:A75,A78,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D78" s="23" t="s">
+      <c r="D78" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E78" s="29" t="s">
+      <c r="E78" s="26" t="s">
         <v>82</v>
       </c>
       <c r="F78" s="9">
         <f>SUMIF(A14:A75,D78,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="G78" s="23" t="s">
+      <c r="G78" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="H78" s="29" t="s">
+      <c r="H78" s="26" t="s">
         <v>84</v>
       </c>
       <c r="I78" s="9">
@@ -3977,30 +3957,30 @@
       <c r="J78" s="2"/>
     </row>
     <row r="79" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="21" t="s">
+      <c r="A79" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B79" s="29" t="s">
+      <c r="B79" s="26" t="s">
         <v>86</v>
       </c>
       <c r="C79" s="9">
         <f>SUMIF(A14:A75,A79,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D79" s="23" t="s">
+      <c r="D79" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="E79" s="29" t="s">
+      <c r="E79" s="26" t="s">
         <v>88</v>
       </c>
       <c r="F79" s="9">
         <f>SUMIF(A14:A75,D79,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="G79" s="23" t="s">
+      <c r="G79" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="H79" s="29" t="s">
+      <c r="H79" s="26" t="s">
         <v>90</v>
       </c>
       <c r="I79" s="9">
@@ -4010,20 +3990,20 @@
       <c r="J79" s="2"/>
     </row>
     <row r="80" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="22" t="s">
+      <c r="A80" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B80" s="29" t="s">
+      <c r="B80" s="26" t="s">
         <v>92</v>
       </c>
       <c r="C80" s="9">
         <f>SUMIF(A14:A75,A80,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D80" s="23" t="s">
+      <c r="D80" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="E80" s="29" t="s">
+      <c r="E80" s="26" t="s">
         <v>94</v>
       </c>
       <c r="F80" s="9">
@@ -4031,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="G80" s="6"/>
-      <c r="H80" s="29" t="s">
+      <c r="H80" s="26" t="s">
         <v>95</v>
       </c>
       <c r="I80" s="9">
@@ -4041,13 +4021,13 @@
       <c r="J80" s="2"/>
     </row>
     <row r="81" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="27" t="s">
+      <c r="A81" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="B81" s="30"/>
+      <c r="B81" s="27"/>
       <c r="C81" s="7"/>
       <c r="D81" s="6"/>
-      <c r="E81" s="30"/>
+      <c r="E81" s="27"/>
       <c r="F81" s="6"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
@@ -4055,20 +4035,20 @@
       <c r="J81" s="2"/>
     </row>
     <row r="82" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="21" t="s">
+      <c r="A82" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="B82" s="29" t="s">
+      <c r="B82" s="26" t="s">
         <v>98</v>
       </c>
       <c r="C82" s="9">
         <f>SUMIF(A14:A75,A82,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D82" s="23" t="s">
+      <c r="D82" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E82" s="31" t="s">
+      <c r="E82" s="28" t="s">
         <v>99</v>
       </c>
       <c r="F82" s="9">
@@ -4081,20 +4061,20 @@
       <c r="J82" s="2"/>
     </row>
     <row r="83" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="21" t="s">
+      <c r="A83" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B83" s="29" t="s">
+      <c r="B83" s="26" t="s">
         <v>100</v>
       </c>
       <c r="C83" s="9">
         <f>SUMIF(A14:A75,A83,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D83" s="23" t="s">
+      <c r="D83" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E83" s="31" t="s">
+      <c r="E83" s="28" t="s">
         <v>101</v>
       </c>
       <c r="F83" s="9">
@@ -4102,7 +4082,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="2"/>
-      <c r="H83" s="29" t="s">
+      <c r="H83" s="26" t="s">
         <v>102</v>
       </c>
       <c r="I83" s="9">
@@ -4112,20 +4092,20 @@
       <c r="J83" s="2"/>
     </row>
     <row r="84" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="22" t="s">
+      <c r="A84" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B84" s="29" t="s">
+      <c r="B84" s="26" t="s">
         <v>104</v>
       </c>
       <c r="C84" s="9">
         <f>SUMIF(A14:A75,A84,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D84" s="23" t="s">
+      <c r="D84" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="E84" s="31" t="s">
+      <c r="E84" s="28" t="s">
         <v>106</v>
       </c>
       <c r="F84" s="9">
@@ -4138,20 +4118,20 @@
       <c r="J84" s="2"/>
     </row>
     <row r="85" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="22" t="s">
+      <c r="A85" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B85" s="31" t="s">
+      <c r="B85" s="28" t="s">
         <v>108</v>
       </c>
       <c r="C85" s="9">
         <f>SUMIF(A14:A75,A85,M14:M75)</f>
         <v>0</v>
       </c>
-      <c r="D85" s="23" t="s">
+      <c r="D85" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="E85" s="31" t="s">
+      <c r="E85" s="28" t="s">
         <v>110</v>
       </c>
       <c r="F85" s="9">
@@ -4164,7 +4144,7 @@
       <c r="J85" s="2"/>
     </row>
     <row r="86" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="27" t="s">
+      <c r="A86" s="24" t="s">
         <v>111</v>
       </c>
       <c r="B86" s="2"/>
@@ -4182,7 +4162,7 @@
     </row>
     <row r="87" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1"/>
-      <c r="B87" s="29" t="s">
+      <c r="B87" s="26" t="s">
         <v>112</v>
       </c>
       <c r="C87" s="9">
@@ -4202,7 +4182,7 @@
     </row>
     <row r="88" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
-      <c r="B88" s="29" t="s">
+      <c r="B88" s="26" t="s">
         <v>113</v>
       </c>
       <c r="C88" s="9">
@@ -4222,7 +4202,7 @@
     </row>
     <row r="89" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
-      <c r="B89" s="29" t="s">
+      <c r="B89" s="26" t="s">
         <v>114</v>
       </c>
       <c r="C89" s="9">
@@ -7746,7 +7726,7 @@
   <protectedRanges>
     <protectedRange sqref="M32" name="Range1"/>
   </protectedRanges>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="B1:M1"/>
     <mergeCell ref="B2:M2"/>
@@ -7760,6 +7740,7 @@
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="I9:J9"/>
+    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>